<commit_message>
KPIs fix and Log in Improved
</commit_message>
<xml_diff>
--- a/teams_info_lucas.xlsx
+++ b/teams_info_lucas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="32">
   <si>
     <t>matchId</t>
   </si>
@@ -104,6 +104,12 @@
   </si>
   <si>
     <t>Leicester</t>
+  </si>
+  <si>
+    <t>Southampton</t>
+  </si>
+  <si>
+    <t>Ipswich</t>
   </si>
 </sst>
 </file>
@@ -461,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1152,13 +1158,13 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>1908653</v>
+        <v>1908636</v>
       </c>
       <c r="C50" t="s">
         <v>3</v>
       </c>
       <c r="D50" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -1166,13 +1172,13 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>1908667</v>
+        <v>1908653</v>
       </c>
       <c r="C51" t="s">
         <v>3</v>
       </c>
       <c r="D51" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -1180,13 +1186,111 @@
         <v>50</v>
       </c>
       <c r="B52">
+        <v>1908667</v>
+      </c>
+      <c r="C52" t="s">
+        <v>3</v>
+      </c>
+      <c r="D52" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="1">
+        <v>51</v>
+      </c>
+      <c r="B53">
         <v>1908669</v>
       </c>
-      <c r="C52" t="s">
-        <v>3</v>
-      </c>
-      <c r="D52" t="s">
+      <c r="C53" t="s">
+        <v>3</v>
+      </c>
+      <c r="D53" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="1">
+        <v>52</v>
+      </c>
+      <c r="B54">
+        <v>1908691</v>
+      </c>
+      <c r="C54" t="s">
+        <v>3</v>
+      </c>
+      <c r="D54" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="1">
+        <v>53</v>
+      </c>
+      <c r="B55">
+        <v>1908700</v>
+      </c>
+      <c r="C55" t="s">
+        <v>3</v>
+      </c>
+      <c r="D55" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="1">
+        <v>54</v>
+      </c>
+      <c r="B56">
+        <v>1908713</v>
+      </c>
+      <c r="C56" t="s">
+        <v>3</v>
+      </c>
+      <c r="D56" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="1">
+        <v>55</v>
+      </c>
+      <c r="B57">
+        <v>1908725</v>
+      </c>
+      <c r="C57" t="s">
+        <v>3</v>
+      </c>
+      <c r="D57" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="1">
+        <v>56</v>
+      </c>
+      <c r="B58">
+        <v>1908733</v>
+      </c>
+      <c r="C58" t="s">
+        <v>3</v>
+      </c>
+      <c r="D58" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="1">
+        <v>57</v>
+      </c>
+      <c r="B59">
+        <v>1908741</v>
+      </c>
+      <c r="C59" t="s">
+        <v>3</v>
+      </c>
+      <c r="D59" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mejorado para que el pdf de individual development se vea bien
</commit_message>
<xml_diff>
--- a/teams_info_lucas.xlsx
+++ b/teams_info_lucas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,7 +576,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1826911</v>
+        <v>1826948</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Oxford</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1826948</v>
+        <v>1826953</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -603,7 +603,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1826953</v>
+        <v>1826963</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1826963</v>
+        <v>1826978</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Luton</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1826978</v>
+        <v>1826982</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Luton</t>
+          <t>Leeds</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1826982</v>
+        <v>1827017</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Swansea</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1827017</v>
+        <v>1827028</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -693,7 +693,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>WBA</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1827028</v>
+        <v>1827051</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>WBA</t>
+          <t>Blackburn</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1827051</v>
+        <v>1827057</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Blackburn</t>
+          <t>Sheff Wed</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1827057</v>
+        <v>1827071</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sheff Wed</t>
+          <t>QPR</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1827071</v>
+        <v>1827076</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>QPR</t>
+          <t>Hull</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1827076</v>
+        <v>1827082</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Bristol City</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1827082</v>
+        <v>1827094</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -801,7 +801,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Portsmouth</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>1827094</v>
+        <v>1827113</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>Burnley</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>1827113</v>
+        <v>1827119</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -837,7 +837,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>Cardiff</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>1827119</v>
+        <v>1827691</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cardiff</t>
+          <t>Preston</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>1827691</v>
+        <v>1827702</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Coventry</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>1827702</v>
+        <v>1827720</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Coventry</t>
+          <t>Sheff Utd</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>1827720</v>
+        <v>1827723</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sheff Utd</t>
+          <t>Derby</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>1827922</v>
+        <v>1827864</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>Hull</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>1908505</v>
+        <v>1827879</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Burnley</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>1908515</v>
+        <v>1827898</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>WBA</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>1908519</v>
+        <v>1827922</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>Swansea</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>1908540</v>
+        <v>1827933</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Blackburn</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>1908546</v>
+        <v>1827955</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Leicester</t>
+          <t>Sheff Wed</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>1908569</v>
+        <v>1908321</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Charlton</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>1908571</v>
+        <v>1908363</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Millwall</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>1908586</v>
+        <v>1908367</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Sheff Wed</t>
+          <t>Blackburn</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>1908631</v>
+        <v>1908387</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>WBA</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>1908636</v>
+        <v>1908389</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Ipswich</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>1908653</v>
+        <v>1908400</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Coventry</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>1908667</v>
+        <v>1908412</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>Southampton</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>1908669</v>
+        <v>1908443</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Blackburn</t>
+          <t>Bristol City</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
         <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>1908691</v>
+        <v>1908455</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1404,7 @@
         <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>1908700</v>
+        <v>1908457</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Southampton</t>
+          <t>Oxford</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>1908713</v>
+        <v>1908464</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Derby</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
         <v>55</v>
       </c>
       <c r="B57" t="n">
-        <v>1908725</v>
+        <v>1908486</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Derby</t>
+          <t>Sheff Utd</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
         <v>56</v>
       </c>
       <c r="B58" t="n">
-        <v>1908733</v>
+        <v>1908505</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Preston</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
         <v>57</v>
       </c>
       <c r="B59" t="n">
-        <v>1908741</v>
+        <v>1908515</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Wrexham</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
         <v>58</v>
       </c>
       <c r="B60" t="n">
-        <v>1908798</v>
+        <v>1908519</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>Birmingham</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
         <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>1908804</v>
+        <v>1908569</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Sheff Wed</t>
+          <t>Norwich</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
         <v>60</v>
       </c>
       <c r="B62" t="n">
-        <v>1908820</v>
+        <v>1908586</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Sheff Wed</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
         <v>61</v>
       </c>
       <c r="B63" t="n">
-        <v>1908834</v>
+        <v>1908607</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Leicester</t>
+          <t>Hull</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
         <v>62</v>
       </c>
       <c r="B64" t="n">
-        <v>1908842</v>
+        <v>1908612</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1584,7 +1584,7 @@
         <v>63</v>
       </c>
       <c r="B65" t="n">
-        <v>1908857</v>
+        <v>1908613</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1593,7 +1593,223 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Charlton</t>
+          <t>Swansea</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="n">
+        <v>1908636</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Hull</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="n">
+        <v>1908667</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Portsmouth</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="n">
+        <v>1908669</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Blackburn</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="n">
+        <v>1908691</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Swansea</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="n">
+        <v>1908700</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1908713</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Preston</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1908725</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Derby</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1908741</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Bristol City</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1908798</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1908804</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Sheff Wed</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" t="n">
+        <v>1908820</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Stoke</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" t="n">
+        <v>1908834</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Leicester</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mejoras al pdf de individual, errores comparacion y filtros
- PDF Individual Development
- Mejorado Errores comparación de jugadores
- Minimo de minutos filtro en partidos
- Toogle por 90 en partidos de futbolista
</commit_message>
<xml_diff>
--- a/teams_info_lucas.xlsx
+++ b/teams_info_lucas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,7 +450,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1826854</v>
+        <v>1908321</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -459,7 +459,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Charlton</t>
         </is>
       </c>
     </row>
@@ -468,7 +468,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1826855</v>
+        <v>1908363</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -477,7 +477,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Derby</t>
+          <t>Millwall</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1826860</v>
+        <v>1908367</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -495,7 +495,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Blackburn</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1826878</v>
+        <v>1908387</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -513,7 +513,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>WBA</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1826881</v>
+        <v>1908389</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -531,7 +531,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Ipswich</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1826896</v>
+        <v>1908412</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -549,7 +549,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sheff Utd</t>
+          <t>Southampton</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1826905</v>
+        <v>1908443</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Coventry</t>
+          <t>Bristol City</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1826948</v>
+        <v>1908455</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1826953</v>
+        <v>1908457</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -603,7 +603,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Oxford</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1826963</v>
+        <v>1908464</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Derby</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1826978</v>
+        <v>1908486</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Luton</t>
+          <t>Sheff Utd</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1826982</v>
+        <v>1908505</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Preston</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1827017</v>
+        <v>1908515</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>Wrexham</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1827028</v>
+        <v>1908519</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -693,7 +693,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>WBA</t>
+          <t>Birmingham</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1827051</v>
+        <v>1908540</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Blackburn</t>
+          <t>Stoke</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1827057</v>
+        <v>1908546</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sheff Wed</t>
+          <t>Leicester</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1827071</v>
+        <v>1908569</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>QPR</t>
+          <t>Norwich</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1827076</v>
+        <v>1908571</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Norwich</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1827082</v>
+        <v>1908586</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Sheff Wed</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1827094</v>
+        <v>1908607</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -801,7 +801,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>Hull</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>1827113</v>
+        <v>1908612</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>QPR</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>1827119</v>
+        <v>1908613</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -837,7 +837,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Cardiff</t>
+          <t>Swansea</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>1827691</v>
+        <v>1908631</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Birmingham</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>1827702</v>
+        <v>1908636</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Coventry</t>
+          <t>Hull</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>1827720</v>
+        <v>1908653</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sheff Utd</t>
+          <t>Millwall</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>1827723</v>
+        <v>1908667</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Derby</t>
+          <t>Portsmouth</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>1827728</v>
+        <v>1908669</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>QPR</t>
+          <t>Blackburn</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>1827739</v>
+        <v>1908691</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Swansea</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>1827754</v>
+        <v>1908700</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Southampton</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>1827761</v>
+        <v>1908713</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -981,7 +981,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Preston</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>1827780</v>
+        <v>1908725</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -999,7 +999,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Derby</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>1827783</v>
+        <v>1908733</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Ipswich</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>1827794</v>
+        <v>1908741</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Bristol City</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>1827805</v>
+        <v>1908798</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>Wrexham</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>1827816</v>
+        <v>1908804</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Sheff Wed</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>1827822</v>
+        <v>1908820</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Cardiff</t>
+          <t>Stoke</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>1827847</v>
+        <v>1908834</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Luton</t>
+          <t>Leicester</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>1827862</v>
+        <v>1908842</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>QPR</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>1827864</v>
+        <v>1908857</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1143,673 +1143,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Hull</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" t="n">
-        <v>1827879</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Burnley</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" t="n">
-        <v>1827898</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>WBA</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" t="n">
-        <v>1827922</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Swansea</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="n">
-        <v>1827933</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Blackburn</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="n">
-        <v>1827955</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Sheff Wed</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="n">
-        <v>1908321</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
           <t>Charlton</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="n">
-        <v>1908363</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Millwall</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="n">
-        <v>1908367</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Blackburn</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="n">
-        <v>1908387</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>WBA</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" t="n">
-        <v>1908389</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Ipswich</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" t="n">
-        <v>1908400</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Coventry</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" t="n">
-        <v>1908412</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Southampton</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" t="n">
-        <v>1908443</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Bristol City</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" t="n">
-        <v>1908455</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Middlesbrough</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" t="n">
-        <v>1908457</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Oxford</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" t="n">
-        <v>1908464</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Derby</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" t="n">
-        <v>1908486</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Sheff Utd</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" t="n">
-        <v>1908505</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Preston</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" t="n">
-        <v>1908515</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Wrexham</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>58</v>
-      </c>
-      <c r="B60" t="n">
-        <v>1908519</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Birmingham</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>59</v>
-      </c>
-      <c r="B61" t="n">
-        <v>1908569</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Norwich</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>60</v>
-      </c>
-      <c r="B62" t="n">
-        <v>1908586</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Sheff Wed</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>61</v>
-      </c>
-      <c r="B63" t="n">
-        <v>1908607</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Hull</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>62</v>
-      </c>
-      <c r="B64" t="n">
-        <v>1908612</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>QPR</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>63</v>
-      </c>
-      <c r="B65" t="n">
-        <v>1908613</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Swansea</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>64</v>
-      </c>
-      <c r="B66" t="n">
-        <v>1908636</v>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Hull</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>65</v>
-      </c>
-      <c r="B67" t="n">
-        <v>1908667</v>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Portsmouth</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>66</v>
-      </c>
-      <c r="B68" t="n">
-        <v>1908669</v>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Blackburn</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>67</v>
-      </c>
-      <c r="B69" t="n">
-        <v>1908691</v>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Swansea</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="n">
-        <v>68</v>
-      </c>
-      <c r="B70" t="n">
-        <v>1908700</v>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Southampton</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="1" t="n">
-        <v>69</v>
-      </c>
-      <c r="B71" t="n">
-        <v>1908713</v>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Preston</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="1" t="n">
-        <v>70</v>
-      </c>
-      <c r="B72" t="n">
-        <v>1908725</v>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Derby</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="1" t="n">
-        <v>71</v>
-      </c>
-      <c r="B73" t="n">
-        <v>1908741</v>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Bristol City</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="1" t="n">
-        <v>72</v>
-      </c>
-      <c r="B74" t="n">
-        <v>1908798</v>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Wrexham</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="1" t="n">
-        <v>73</v>
-      </c>
-      <c r="B75" t="n">
-        <v>1908804</v>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Sheff Wed</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="1" t="n">
-        <v>74</v>
-      </c>
-      <c r="B76" t="n">
-        <v>1908820</v>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Stoke</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="1" t="n">
-        <v>75</v>
-      </c>
-      <c r="B77" t="n">
-        <v>1908834</v>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Leicester</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pdf de comparison realizado y empezado card players
</commit_message>
<xml_diff>
--- a/teams_info_lucas.xlsx
+++ b/teams_info_lucas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,7 +450,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1826854</v>
+        <v>1908321</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -459,7 +459,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Charlton</t>
         </is>
       </c>
     </row>
@@ -468,7 +468,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1826855</v>
+        <v>1908363</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -477,7 +477,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Derby</t>
+          <t>Millwall</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1826860</v>
+        <v>1908367</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -495,7 +495,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Blackburn</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1826878</v>
+        <v>1908387</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -513,7 +513,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>WBA</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1826881</v>
+        <v>1908389</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -531,7 +531,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Ipswich</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1826896</v>
+        <v>1908412</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -549,7 +549,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sheff Utd</t>
+          <t>Southampton</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1826905</v>
+        <v>1908443</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Coventry</t>
+          <t>Bristol City</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1826911</v>
+        <v>1908455</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1826948</v>
+        <v>1908457</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1826953</v>
+        <v>1908464</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Derby</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1826963</v>
+        <v>1908486</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Sheff Utd</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1826978</v>
+        <v>1908505</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Luton</t>
+          <t>Preston</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1826982</v>
+        <v>1908515</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Wrexham</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1827017</v>
+        <v>1908519</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -693,7 +693,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>Birmingham</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1827028</v>
+        <v>1908540</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>WBA</t>
+          <t>Stoke</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1827051</v>
+        <v>1908546</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Blackburn</t>
+          <t>Leicester</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1827057</v>
+        <v>1908569</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sheff Wed</t>
+          <t>Norwich</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1827071</v>
+        <v>1908571</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>QPR</t>
+          <t>Norwich</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1827076</v>
+        <v>1908586</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Sheff Wed</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1827082</v>
+        <v>1908607</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -801,7 +801,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Hull</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>1827094</v>
+        <v>1908612</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>QPR</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>1827113</v>
+        <v>1908613</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -837,7 +837,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>Swansea</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>1827119</v>
+        <v>1908631</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cardiff</t>
+          <t>Birmingham</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>1827691</v>
+        <v>1908636</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Hull</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>1827702</v>
+        <v>1908653</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Coventry</t>
+          <t>Millwall</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>1827720</v>
+        <v>1908667</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sheff Utd</t>
+          <t>Portsmouth</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>1827728</v>
+        <v>1908669</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>QPR</t>
+          <t>Blackburn</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>1827739</v>
+        <v>1908691</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Swansea</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>1827754</v>
+        <v>1908700</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Southampton</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>1827761</v>
+        <v>1908713</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -981,7 +981,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Preston</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>1827780</v>
+        <v>1908725</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -999,7 +999,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Derby</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>1827783</v>
+        <v>1908733</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Ipswich</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>1827794</v>
+        <v>1908741</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Bristol City</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>1827805</v>
+        <v>1908764</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>WBA</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>1827816</v>
+        <v>1908798</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Wrexham</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>1827822</v>
+        <v>1908804</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Cardiff</t>
+          <t>Sheff Wed</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>1827847</v>
+        <v>1908820</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Luton</t>
+          <t>Stoke</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>1827862</v>
+        <v>1908834</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Leicester</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>1827922</v>
+        <v>1908842</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>QPR</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>1908505</v>
+        <v>1908857</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Charlton</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>1908515</v>
+        <v>1908865</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>Oxford</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>1908519</v>
+        <v>1908881</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1197,403 +1197,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Birmingham</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="n">
-        <v>1908540</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Stoke</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="n">
-        <v>1908546</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Leicester</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="n">
-        <v>1908569</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Norwich</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="n">
-        <v>1908571</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Norwich</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="n">
-        <v>1908586</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Sheff Wed</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="n">
-        <v>1908631</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Birmingham</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" t="n">
-        <v>1908636</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Hull</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" t="n">
-        <v>1908653</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Millwall</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" t="n">
-        <v>1908667</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Portsmouth</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" t="n">
-        <v>1908669</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Blackburn</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" t="n">
-        <v>1908691</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Swansea</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" t="n">
-        <v>1908700</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Southampton</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" t="n">
-        <v>1908713</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Preston</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" t="n">
-        <v>1908725</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Derby</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" t="n">
-        <v>1908733</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Ipswich</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" t="n">
-        <v>1908741</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Bristol City</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>58</v>
-      </c>
-      <c r="B60" t="n">
-        <v>1908798</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Wrexham</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>59</v>
-      </c>
-      <c r="B61" t="n">
-        <v>1908804</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Sheff Wed</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>60</v>
-      </c>
-      <c r="B62" t="n">
-        <v>1908820</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Stoke</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>61</v>
-      </c>
-      <c r="B63" t="n">
-        <v>1908834</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Leicester</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>62</v>
-      </c>
-      <c r="B64" t="n">
-        <v>1908842</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>QPR</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>63</v>
-      </c>
-      <c r="B65" t="n">
-        <v>1908857</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Charlton</t>
+          <t>Sheff Utd</t>
         </is>
       </c>
     </row>

</xml_diff>